<commit_message>
limpeza de texto, relatorios e documentacao
</commit_message>
<xml_diff>
--- a/analise_forum/resultados_analise.xlsx
+++ b/analise_forum/resultados_analise.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -430,10 +430,15 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>mensagem_limpa</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Emocao</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Confianca</t>
         </is>
@@ -450,10 +455,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>O portal acadêmico está fora do ar de novo na hora da entrega, que ódio!</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>anger</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.8893</v>
       </c>
     </row>
@@ -468,10 +478,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Achei a discussão do grupo de hoje muito produtiva e esclarecedora.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>admiration</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.8189</v>
       </c>
     </row>
@@ -486,10 +501,15 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Estou completamente perdido com os prazos dessa matéria...</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>disappointment</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.8257</v>
       </c>
     </row>
@@ -499,16 +519,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Finalmente consegui entender a lógica do projeto!</t>
+          <t>O portal &lt;a href='link'&gt;portal.univ.edu&lt;/a&gt; tá travado de novo!! @suporte resolve isso por favor, preciso entregar o TP 😡 https://erro.com/404</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>approval</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0.5296</v>
+          <t xml:space="preserve">O portal portal.univ.edu tá travado de novo!! resolve isso por favor, preciso entregar o TP </t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9638</v>
       </c>
     </row>
     <row r="6">
@@ -517,16 +542,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Muito frustrado com a falta de retorno sobre as dúvidas do trabalho.</t>
+          <t>**Excelente** a aula de hoje! Os slides sobre *Processamento de Linguagem Natural* ajudaram bastante a esclarecer as dúvidas. Valeu @caio_monitor 🙌✨</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>annoyance</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>0.6987</v>
+          <t xml:space="preserve">Excelente a aula de hoje! Os slides sobre Processamento de Linguagem Natural ajudaram bastante a esclarecer as dúvidas. Valeu </t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>gratitude</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9540999999999999</v>
       </c>
     </row>
     <row r="7">
@@ -535,16 +565,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Que notícia excelente! Adiaram a data final do projeto.</t>
+          <t>estou   totalmente   perdido   no   trabalho...   alguém   pode   me   ajudar???    não entendi o enunciado da questão 3 #ajuda</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>admiration</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>0.9159</v>
+          <t>estou totalmente perdido no trabalho... alguém pode me ajudar??? não entendi o enunciado da questão 3 ajuda</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>confusion</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.8275</v>
       </c>
     </row>
     <row r="8">
@@ -553,16 +588,21 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Não sei se vou conseguir entregar tudo, bateu o desespero total.</t>
+          <t>Gente, adiaram a data de entrega para a próxima sexta!! 🎉🎉🎉 Vejam o aviso oficial em www.forum.edu/avisos_oficiais @todos</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>disappointment</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0.679</v>
+          <t>Gente, adiaram a data de entrega para a próxima sexta!!  Vejam o aviso oficial em</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>0.9295</v>
       </c>
     </row>
     <row r="9">
@@ -571,16 +611,21 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ótima explicação na aula de hoje, me ajudou bastante!</t>
+          <t>@maria_123 acho que vou reprovar nessa matéria... tirei nota muito baixa no teste e tô bem desanimado 😔</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>admiration</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>0.9845</v>
+          <t xml:space="preserve">acho que vou reprovar nessa matéria... tirei nota muito baixa no teste e tô bem desanimado </t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>sadness</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.7847</v>
       </c>
     </row>
     <row r="10">
@@ -589,34 +634,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Que vontade de largar a escola</t>
+          <t>Alguém sabe se o laboratório de IA vai estar aberto amanhã à tarde? Preciso testar um script `python main.py` lá.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>neutral</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>0.6172</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Vou abandonar os estudos</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>sadness</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>0.714</v>
+          <t>Alguém sabe se o laboratório de IA vai estar aberto amanhã à tarde? Preciso testar um script python main.py lá.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>curiosity</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0.9381</v>
       </c>
     </row>
   </sheetData>
@@ -630,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -648,61 +680,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>admiration</t>
+          <t>neutral</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>30</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>disappointment</t>
+          <t>anger</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>anger</t>
+          <t>admiration</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>disappointment</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>annoyance</t>
+          <t>gratitude</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>neutral</t>
+          <t>confusion</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="8">
@@ -712,7 +744,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>curiosity</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>11.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>